<commit_message>
Log history Done Problem Refresh fixed
</commit_message>
<xml_diff>
--- a/SMI-Excels/TR/TR-DIV_V2.xlsx
+++ b/SMI-Excels/TR/TR-DIV_V2.xlsx
@@ -1,43 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alaab\Desktop\SMI-Excels\TR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\DEC\SMI-Excels\TR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231A26C1-1A79-49FA-98AF-90CD101AFB15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB11D3BE-C44E-4845-821C-CF11569A8427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{91D9DAF5-8B02-4F39-AF66-D6771BE24E02}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{91D9DAF5-8B02-4F39-AF66-D6771BE24E02}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
     <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Feuil2!$A$1:$G$29</definedName>
+  </definedNames>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="113">
   <si>
     <t>NbrEcritures</t>
   </si>
@@ -343,6 +335,39 @@
   </si>
   <si>
     <t>Contrôle d’existence dans le référentiel des pays de la BCT</t>
+  </si>
+  <si>
+    <t>023</t>
+  </si>
+  <si>
+    <t>1633896D</t>
+  </si>
+  <si>
+    <t>FHC ABIR</t>
+  </si>
+  <si>
+    <t>Ben Jaber</t>
+  </si>
+  <si>
+    <t>Alaa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FHC abir </t>
+  </si>
+  <si>
+    <t>0625</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>12345678912345600000</t>
+  </si>
+  <si>
+    <t>000001</t>
+  </si>
+  <si>
+    <t>R</t>
   </si>
 </sst>
 </file>
@@ -422,7 +447,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -439,6 +464,11 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20 % - Accent1" xfId="1" builtinId="30"/>
@@ -775,38 +805,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19972087-0EB2-4947-94D4-9ED78A20123B}">
-  <dimension ref="A1:AQ1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AQ2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="8" width="14.109375" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.08984375" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.36328125" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.36328125" customWidth="1"/>
+    <col min="8" max="8" width="14.08984375" customWidth="1"/>
+    <col min="9" max="9" width="16.36328125" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="12.21875" customWidth="1"/>
-    <col min="12" max="12" width="13.44140625" customWidth="1"/>
-    <col min="13" max="13" width="20.44140625" customWidth="1"/>
-    <col min="14" max="14" width="35.21875" customWidth="1"/>
+    <col min="11" max="11" width="12.1796875" customWidth="1"/>
+    <col min="12" max="12" width="13.453125" customWidth="1"/>
+    <col min="13" max="13" width="20.453125" customWidth="1"/>
+    <col min="14" max="14" width="35.1796875" customWidth="1"/>
     <col min="16" max="16" width="12" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.90625" style="7"/>
     <col min="27" max="27" width="8" customWidth="1"/>
-    <col min="28" max="28" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="21" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="6" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -815,7 +846,7 @@
       <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -872,7 +903,7 @@
       <c r="X1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="6" t="s">
         <v>9</v>
       </c>
       <c r="Z1" s="1" t="s">
@@ -881,7 +912,7 @@
       <c r="AA1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="6" t="s">
         <v>24</v>
       </c>
       <c r="AC1" s="1" t="s">
@@ -902,6 +933,86 @@
       <c r="AP1" s="1"/>
       <c r="AQ1" s="1"/>
     </row>
+    <row r="2" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2026</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D2">
+        <v>2026</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H2" t="s">
+        <v>104</v>
+      </c>
+      <c r="I2" t="s">
+        <v>112</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>2026</v>
+      </c>
+      <c r="L2" s="8">
+        <v>46023</v>
+      </c>
+      <c r="M2">
+        <v>1100</v>
+      </c>
+      <c r="N2">
+        <v>934</v>
+      </c>
+      <c r="O2">
+        <v>3700</v>
+      </c>
+      <c r="P2">
+        <v>788</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>109</v>
+      </c>
+      <c r="R2">
+        <v>10</v>
+      </c>
+      <c r="S2">
+        <v>1</v>
+      </c>
+      <c r="T2" t="s">
+        <v>105</v>
+      </c>
+      <c r="U2" t="s">
+        <v>106</v>
+      </c>
+      <c r="V2">
+        <v>788</v>
+      </c>
+      <c r="W2" t="s">
+        <v>107</v>
+      </c>
+      <c r="Y2" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="AB2" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="AC2">
+        <v>788</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -909,15 +1020,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36D8DB9C-3803-4ECD-83B3-057AAB8EAD31}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.21875" customWidth="1"/>
+    <col min="1" max="1" width="24.1796875" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="5" width="39.6640625" customWidth="1"/>
+    <col min="5" max="5" width="39.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>26</v>
       </c>
@@ -940,7 +1052,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>33</v>
       </c>
@@ -961,7 +1073,7 @@
       </c>
       <c r="G2" s="3"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>38</v>
       </c>
@@ -982,7 +1094,7 @@
       </c>
       <c r="G3" s="3"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>42</v>
       </c>
@@ -1001,7 +1113,7 @@
       </c>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
@@ -1022,7 +1134,7 @@
       </c>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>1</v>
       </c>
@@ -1043,7 +1155,7 @@
       </c>
       <c r="G6" s="3"/>
     </row>
-    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>0</v>
       </c>
@@ -1064,7 +1176,7 @@
       </c>
       <c r="G7" s="3"/>
     </row>
-    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>2</v>
       </c>
@@ -1085,7 +1197,7 @@
       </c>
       <c r="G8" s="3"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
@@ -1104,7 +1216,7 @@
       </c>
       <c r="G9" s="3"/>
     </row>
-    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
@@ -1125,7 +1237,7 @@
       </c>
       <c r="G10" s="3"/>
     </row>
-    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>16</v>
       </c>
@@ -1146,7 +1258,7 @@
       </c>
       <c r="G11" s="3"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>4</v>
       </c>
@@ -1167,7 +1279,7 @@
       </c>
       <c r="G12" s="3"/>
     </row>
-    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>5</v>
       </c>
@@ -1188,7 +1300,7 @@
       </c>
       <c r="G13" s="3"/>
     </row>
-    <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>6</v>
       </c>
@@ -1209,7 +1321,7 @@
       </c>
       <c r="G14" s="3"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>10</v>
       </c>
@@ -1230,7 +1342,7 @@
       </c>
       <c r="G15" s="3"/>
     </row>
-    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>3</v>
       </c>
@@ -1251,7 +1363,7 @@
       </c>
       <c r="G16" s="3"/>
     </row>
-    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>25</v>
       </c>
@@ -1272,7 +1384,7 @@
       </c>
       <c r="G17" s="3"/>
     </row>
-    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>13</v>
       </c>
@@ -1293,7 +1405,7 @@
       </c>
       <c r="G18" s="3"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>17</v>
       </c>
@@ -1314,7 +1426,7 @@
       </c>
       <c r="G19" s="3"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>8</v>
       </c>
@@ -1335,7 +1447,7 @@
       </c>
       <c r="G20" s="3"/>
     </row>
-    <row r="21" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>18</v>
       </c>
@@ -1356,7 +1468,7 @@
       </c>
       <c r="G21" s="3"/>
     </row>
-    <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
         <v>86</v>
       </c>
@@ -1377,7 +1489,7 @@
       </c>
       <c r="G22" s="3"/>
     </row>
-    <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>19</v>
       </c>
@@ -1398,7 +1510,7 @@
       </c>
       <c r="G23" s="3"/>
     </row>
-    <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
         <v>20</v>
       </c>
@@ -1419,7 +1531,7 @@
       </c>
       <c r="G24" s="3"/>
     </row>
-    <row r="25" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>21</v>
       </c>
@@ -1440,7 +1552,7 @@
       </c>
       <c r="G25" s="3"/>
     </row>
-    <row r="26" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>23</v>
       </c>
@@ -1461,7 +1573,7 @@
       </c>
       <c r="G26" s="3"/>
     </row>
-    <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>22</v>
       </c>
@@ -1482,7 +1594,7 @@
       </c>
       <c r="G27" s="3"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>24</v>
       </c>
@@ -1501,7 +1613,7 @@
       </c>
       <c r="G28" s="3"/>
     </row>
-    <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>11</v>
       </c>
@@ -1522,6 +1634,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G29" xr:uid="{36D8DB9C-3803-4ECD-83B3-057AAB8EAD31}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="O"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>